<commit_message>
Update Comparacion de tiempos.xlsx
</commit_message>
<xml_diff>
--- a/Comparacion de tiempos.xlsx
+++ b/Comparacion de tiempos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/7789b221288dc1f1/Documentos/GitHub/sort-compare/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="258" documentId="11_AD4D2F04E46CFB4ACB3E20A86552CEA2683EDF1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AD0EF224-FB0A-4892-AE23-C8431B799E72}"/>
+  <xr:revisionPtr revIDLastSave="265" documentId="11_AD4D2F04E46CFB4ACB3E20A86552CEA2683EDF1F" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9BEC4FC-DA8D-4A3D-A116-7B9ACC182F09}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -79,9 +79,9 @@
     <numFmt numFmtId="164" formatCode="0.00000"/>
     <numFmt numFmtId="165" formatCode="0.000000"/>
     <numFmt numFmtId="166" formatCode="0.0000000"/>
-    <numFmt numFmtId="169" formatCode="0.0000"/>
+    <numFmt numFmtId="167" formatCode="0.0000"/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,6 +91,14 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -299,6 +307,21 @@
     <xf numFmtId="165" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -314,22 +337,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="1" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -626,36 +634,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="31" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18" t="s">
+      <c r="B1" s="33" t="s">
         <v>8</v>
       </c>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="18" t="s">
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
+      <c r="F1" s="34"/>
+      <c r="G1" s="35"/>
+      <c r="H1" s="33" t="s">
         <v>9</v>
       </c>
-      <c r="I1" s="19"/>
-      <c r="J1" s="19"/>
-      <c r="K1" s="19"/>
-      <c r="L1" s="19"/>
-      <c r="M1" s="20"/>
-      <c r="N1" s="18" t="s">
+      <c r="I1" s="34"/>
+      <c r="J1" s="34"/>
+      <c r="K1" s="34"/>
+      <c r="L1" s="34"/>
+      <c r="M1" s="35"/>
+      <c r="N1" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="O1" s="19"/>
-      <c r="P1" s="19"/>
-      <c r="Q1" s="19"/>
-      <c r="R1" s="19"/>
-      <c r="S1" s="20"/>
+      <c r="O1" s="34"/>
+      <c r="P1" s="34"/>
+      <c r="Q1" s="34"/>
+      <c r="R1" s="34"/>
+      <c r="S1" s="35"/>
     </row>
     <row r="2" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="17"/>
+      <c r="A2" s="32"/>
       <c r="B2" s="2">
         <v>1</v>
       </c>
@@ -715,38 +723,38 @@
       <c r="A3" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="23">
+      <c r="B3" s="18">
         <v>5.4836273193359299E-6</v>
       </c>
-      <c r="C3" s="24">
+      <c r="C3" s="19">
         <v>5.7220458984375E-6</v>
       </c>
-      <c r="D3" s="24">
+      <c r="D3" s="19">
         <v>5.00679016113281E-6</v>
       </c>
-      <c r="E3" s="24">
+      <c r="E3" s="19">
         <v>4.5299530029296799E-6</v>
       </c>
-      <c r="F3" s="25">
+      <c r="F3" s="20">
         <v>5.7220458984375E-6</v>
       </c>
-      <c r="G3" s="21">
+      <c r="G3" s="16">
         <f>AVERAGE(B3:F3)</f>
         <v>5.2928924560546839E-6</v>
       </c>
-      <c r="H3" s="32">
+      <c r="H3" s="26">
         <v>1.6619682312011701E-2</v>
       </c>
-      <c r="I3" s="36">
+      <c r="I3" s="30">
         <v>1.5666246414184501E-2</v>
       </c>
-      <c r="J3" s="36">
+      <c r="J3" s="30">
         <v>1.4676809310912999E-2</v>
       </c>
-      <c r="K3" s="36">
+      <c r="K3" s="30">
         <v>1.5172004699707E-2</v>
       </c>
-      <c r="L3" s="36">
+      <c r="L3" s="30">
         <v>1.52561664581298E-2</v>
       </c>
       <c r="M3" s="12">
@@ -780,35 +788,35 @@
       <c r="B4" s="8">
         <v>5.96046447753906E-6</v>
       </c>
-      <c r="C4" s="26">
+      <c r="C4" s="9">
         <v>7.1525573730468699E-6</v>
       </c>
-      <c r="D4" s="26">
+      <c r="D4" s="9">
         <v>6.1988830566406199E-6</v>
       </c>
-      <c r="E4" s="26">
+      <c r="E4" s="9">
         <v>6.91413879394531E-6</v>
       </c>
-      <c r="F4" s="27">
+      <c r="F4" s="21">
         <v>7.1525573730468699E-6</v>
       </c>
-      <c r="G4" s="21">
+      <c r="G4" s="16">
         <f t="shared" ref="G4:G8" si="0">AVERAGE(B4:F4)</f>
         <v>6.6757202148437458E-6</v>
       </c>
-      <c r="H4" s="32">
+      <c r="H4" s="26">
         <v>1.5654802322387602E-2</v>
       </c>
-      <c r="I4" s="36">
+      <c r="I4" s="30">
         <v>1.5982389450073201E-2</v>
       </c>
-      <c r="J4" s="36">
+      <c r="J4" s="30">
         <v>1.52795314788818E-2</v>
       </c>
-      <c r="K4" s="36">
+      <c r="K4" s="30">
         <v>1.5976905822753899E-2</v>
       </c>
-      <c r="L4" s="36">
+      <c r="L4" s="30">
         <v>1.5918970108032199E-2</v>
       </c>
       <c r="M4" s="12">
@@ -842,35 +850,35 @@
       <c r="B5" s="8">
         <v>6.91413879394531E-6</v>
       </c>
-      <c r="C5" s="26">
+      <c r="C5" s="9">
         <v>1.5497207641601502E-5</v>
       </c>
-      <c r="D5" s="26">
+      <c r="D5" s="9">
         <v>6.67572021484375E-6</v>
       </c>
-      <c r="E5" s="26">
+      <c r="E5" s="9">
         <v>6.67572021484375E-6</v>
       </c>
-      <c r="F5" s="27">
+      <c r="F5" s="21">
         <v>1.52587890625E-5</v>
       </c>
-      <c r="G5" s="21">
+      <c r="G5" s="16">
         <f t="shared" si="0"/>
         <v>1.0204315185546861E-5</v>
       </c>
-      <c r="H5" s="36">
+      <c r="H5" s="30">
         <v>3.4366607666015597E-2</v>
       </c>
-      <c r="I5" s="36">
+      <c r="I5" s="30">
         <v>3.2799720764160101E-2</v>
       </c>
-      <c r="J5" s="36">
+      <c r="J5" s="30">
         <v>3.1974077224731397E-2</v>
       </c>
-      <c r="K5" s="36">
+      <c r="K5" s="30">
         <v>3.2957792282104402E-2</v>
       </c>
-      <c r="L5" s="36">
+      <c r="L5" s="30">
         <v>4.3374538421630797E-2</v>
       </c>
       <c r="M5" s="12">
@@ -904,54 +912,54 @@
       <c r="B6" s="8">
         <v>1.28746032714843E-5</v>
       </c>
-      <c r="C6" s="26">
+      <c r="C6" s="9">
         <v>1.2397766113281199E-5</v>
       </c>
-      <c r="D6" s="26">
+      <c r="D6" s="9">
         <v>1.71661376953125E-5</v>
       </c>
-      <c r="E6" s="26">
+      <c r="E6" s="9">
         <v>1.38282775878906E-5</v>
       </c>
-      <c r="F6" s="27">
+      <c r="F6" s="21">
         <v>1.31130218505859E-5</v>
       </c>
-      <c r="G6" s="21">
+      <c r="G6" s="16">
         <f t="shared" si="0"/>
         <v>1.3875961303710899E-5</v>
       </c>
-      <c r="H6" s="36">
+      <c r="H6" s="30">
         <v>1.5618801116943301E-3</v>
       </c>
-      <c r="I6" s="36">
+      <c r="I6" s="30">
         <v>1.3227462768554601E-3</v>
       </c>
-      <c r="J6" s="36">
+      <c r="J6" s="30">
         <v>1.32632255554199E-3</v>
       </c>
-      <c r="K6" s="36">
+      <c r="K6" s="30">
         <v>1.2161731719970701E-3</v>
       </c>
-      <c r="L6" s="36">
+      <c r="L6" s="30">
         <v>1.2781620025634701E-3</v>
       </c>
       <c r="M6" s="12">
         <f t="shared" si="1"/>
         <v>1.3410568237304638E-3</v>
       </c>
-      <c r="N6" s="35">
+      <c r="N6" s="29">
         <v>9.2754602432250893E-2</v>
       </c>
-      <c r="O6" s="35">
+      <c r="O6" s="29">
         <v>0.10171556472778299</v>
       </c>
-      <c r="P6" s="35">
+      <c r="P6" s="29">
         <v>9.4923019409179604E-2</v>
       </c>
-      <c r="Q6" s="35">
+      <c r="Q6" s="29">
         <v>9.4741582870483398E-2</v>
       </c>
-      <c r="R6" s="35">
+      <c r="R6" s="29">
         <v>9.6983671188354395E-2</v>
       </c>
       <c r="S6" s="10">
@@ -966,54 +974,54 @@
       <c r="B7" s="8">
         <v>4.4898986816406198E-3</v>
       </c>
-      <c r="C7" s="26">
+      <c r="C7" s="9">
         <v>7.62939453125E-6</v>
       </c>
-      <c r="D7" s="26">
+      <c r="D7" s="9">
         <v>5.2452087402343699E-6</v>
       </c>
-      <c r="E7" s="26">
+      <c r="E7" s="9">
         <v>5.7220458984375E-6</v>
       </c>
-      <c r="F7" s="27">
+      <c r="F7" s="21">
         <v>5.96046447753906E-6</v>
       </c>
-      <c r="G7" s="21">
+      <c r="G7" s="16">
         <f t="shared" si="0"/>
         <v>9.028911590576161E-4</v>
       </c>
-      <c r="H7" s="32">
+      <c r="H7" s="26">
         <v>7.09295272827148E-4</v>
       </c>
-      <c r="I7" s="36">
+      <c r="I7" s="30">
         <v>2.4223327636718701E-4</v>
       </c>
-      <c r="J7" s="36">
+      <c r="J7" s="30">
         <v>2.4890899658203098E-4</v>
       </c>
-      <c r="K7" s="36">
+      <c r="K7" s="30">
         <v>2.3365020751953101E-4</v>
       </c>
-      <c r="L7" s="36">
+      <c r="L7" s="30">
         <v>2.1934509277343701E-4</v>
       </c>
       <c r="M7" s="12">
         <f t="shared" si="1"/>
         <v>3.3068656921386686E-4</v>
       </c>
-      <c r="N7" s="29">
+      <c r="N7" s="23">
         <v>1.67205333709716E-2</v>
       </c>
-      <c r="O7" s="35">
+      <c r="O7" s="29">
         <v>2.0035505294799801E-2</v>
       </c>
-      <c r="P7" s="35">
+      <c r="P7" s="29">
         <v>1.7355442047119099E-2</v>
       </c>
-      <c r="Q7" s="35">
+      <c r="Q7" s="29">
         <v>1.9801378250122001E-2</v>
       </c>
-      <c r="R7" s="35">
+      <c r="R7" s="29">
         <v>2.09097862243652E-2</v>
       </c>
       <c r="S7" s="10">
@@ -1037,45 +1045,45 @@
       <c r="E8" s="15">
         <v>2.5033950805664002E-5</v>
       </c>
-      <c r="F8" s="28">
+      <c r="F8" s="22">
         <v>2.5272369384765601E-5</v>
       </c>
-      <c r="G8" s="22">
+      <c r="G8" s="17">
         <f t="shared" si="0"/>
         <v>1.9264221191406178E-5</v>
       </c>
-      <c r="H8" s="33">
+      <c r="H8" s="27">
         <v>9.6654891967773405E-4</v>
       </c>
-      <c r="I8" s="34">
+      <c r="I8" s="28">
         <v>9.3674659729003895E-4</v>
       </c>
-      <c r="J8" s="34">
+      <c r="J8" s="28">
         <v>9.2482566833495996E-4</v>
       </c>
-      <c r="K8" s="34">
+      <c r="K8" s="28">
         <v>9.3317031860351497E-4</v>
       </c>
-      <c r="L8" s="34">
+      <c r="L8" s="28">
         <v>9.3102455139160102E-4</v>
       </c>
       <c r="M8" s="13">
         <f t="shared" si="1"/>
         <v>9.3846321105956984E-4</v>
       </c>
-      <c r="N8" s="30">
+      <c r="N8" s="24">
         <v>7.0123672485351493E-2</v>
       </c>
-      <c r="O8" s="31">
+      <c r="O8" s="25">
         <v>7.1588277816772405E-2</v>
       </c>
-      <c r="P8" s="31">
+      <c r="P8" s="25">
         <v>7.3649644851684501E-2</v>
       </c>
-      <c r="Q8" s="31">
+      <c r="Q8" s="25">
         <v>7.2632312774658203E-2</v>
       </c>
-      <c r="R8" s="31">
+      <c r="R8" s="25">
         <v>7.4522256851196206E-2</v>
       </c>
       <c r="S8" s="11">
@@ -1084,29 +1092,19 @@
       </c>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="9">
-        <v>7.0123672485351493E-2</v>
-      </c>
+      <c r="B10" s="36"/>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="9">
-        <v>7.1588277816772405E-2</v>
-      </c>
+      <c r="B11" s="36"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B12" s="9">
-        <v>7.3649644851684501E-2</v>
-      </c>
+      <c r="B12" s="36"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B13" s="9">
-        <v>7.2632312774658203E-2</v>
-      </c>
+      <c r="B13" s="36"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="9">
-        <v>7.4522256851196206E-2</v>
-      </c>
+      <c r="B14" s="36"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>